<commit_message>
feat(memo-90): upgrade บันทึกข้อความ_90_วัน to Ref. 90-day 17pt uniform standard and save reference
</commit_message>
<xml_diff>
--- a/frontend/static/docs/บันทึกข้อความ_90_วัน_Rebuild_Thai.xlsx
+++ b/frontend/static/docs/บันทึกข้อความ_90_วัน_Rebuild_Thai.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,17 +27,21 @@
     </font>
     <font>
       <name val="TH Sarabun PSK"/>
-      <b val="1"/>
-      <sz val="18"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="TH Sarabun PSK"/>
       <b val="1"/>
-      <sz val="12"/>
+      <sz val="24"/>
     </font>
     <font>
       <name val="TH Sarabun PSK"/>
-      <sz val="12"/>
+      <b val="1"/>
+      <sz val="17"/>
+    </font>
+    <font>
+      <name val="TH Sarabun PSK"/>
+      <sz val="17"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,15 +64,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,121 +448,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B4:E18"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="4">
-      <c r="C4" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>( สำเนาคู่ฉบับ )</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>บันทึกข้อความ</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="2" t="inlineStr">
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>ส่วนราชการ</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>ป.๔ พัน.๔ ร้อย.๒  (โทร ๓๑๑๙๓)</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="2" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>ที่</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>กห ๐๔๘๓.๑.๔.๑/       วันที่            ก.ย. ๖๙</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>กห ๐๔๘๓.๑.๔.๑/</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>วันที่</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>ก.ย. ๖๙</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>เรื่อง</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>ขอส่งใบติดตามใบส่งซ่อมเกิน ๙๐ วัน</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="2" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>เรียน</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>ผบ.ป.๔ พัน.๔ (ผ่าน หมู่ส่งกำลังบำรุงฯ)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>อ้างถึง</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>๑. ระเบียบ ทบ. ว่าด้วยส่งกำลังสิ่งอุปกรณ์ประเภท ๒ และ ๔ พ.ศ. ๒๕๓๔</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="2" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>สิ่งที่ส่งมาด้วย</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>ใบติดตามใบส่งซ่อม สิ่งอุปกรณ์ ทบ.๔๐๐-๐๗๑   จำนวน  ๑  ฉบับ</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>ป.๔ พัน.๔ ร้อย.๒ ขอติดตามใบส่งซ่อมเกิน ๙๐ วัน สิ่งอุปกรณ์ของ ปบค.๙๕ ขนาด ๑๐๕ มม. เอ็ม.๑๐๑ เอ.๑ ปรับปรุง รายละเอียดตามสิ่งที่ส่งมาด้วย</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="3" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>จึงเรียนมาเพื่อกรุณาพิจารณา</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>ร.อ.
-(กฤติน  นราพงษ์)
-ผบ.ป.๔ พัน.๔ ร้อย.๒</t>
+    <row r="16">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>ร.อ.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>(กฤติน  นราพงษ์)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>ผบ.ป.๔ พัน.๔ ร้อย.๒</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>จ.ส.อ.</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>ร่าง/ตรวจ    ก.ย. ๖๙</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>ส.อ. อวิวัฒน์ฯ</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>พิมพ์/ทาน  ๑๘    ก.ย. ๖๙</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B3:D3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>